<commit_message>
Gaia's palette, a warm sun, a diorama orbit, visible rain, one post pass
Every colour comes from one PAL block. ACES tone mapping with a warm sun
and a cool-warm hemisphere. Pitch held between 40 and 62 degrees. Rain is
a translucent shaft from ground to cloud; ground under film water darkens
and blues. A single full-screen shader does tilt-shift, grade and vignette,
toggled from View as Diorama. Screenshots at radius 12 and 36 in design/.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X15nfPExS7vTWJ6rHqpTfb
</commit_message>
<xml_diff>
--- a/design/mechanics.xlsx
+++ b/design/mechanics.xlsx
@@ -747,9 +747,9 @@
           <t>world</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>next</t>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -762,11 +762,15 @@
           <t>A shore greens in about one Season, not one Moon; a Year covers about 50 hexes from one seed.</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>12-hex shore greens over 56 ticks (was 5); alive every 10 ticks 3 5 7 9 11 12</t>
+        </is>
+      </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Without this a seed covers the pot in one Season once the world breathes.</t>
+          <t>Commit "Life keeps its own clock". Without this a seed covers the pot in one Season once the world breathes.</t>
         </is>
       </c>
     </row>
@@ -794,9 +798,9 @@
           <t>game</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>next</t>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -809,11 +813,15 @@
           <t>Watching is the fun; nobody waits; nobody is rushed. One cloud fills a 7-hex 2-deep bowl in one Season.</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>headless: 5 ticks in 2.6 s at 1x, +40 in 2.1 s at 10x, 0 while paused; clock shows Year/Season</t>
+        </is>
+      </c>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Replaces the Moon-per-action idea from design v0.1. Pause is a courtesy, never required.</t>
+          <t>Mana not yet: actions are free until step 6. Replaces the Moon-per-action idea from design v0.1. Pause is a courtesy, never required.</t>
         </is>
       </c>
     </row>
@@ -841,9 +849,9 @@
           <t>presentation</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>next</t>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -856,11 +864,15 @@
           <t>A stranger reads lake, river, hill, life without a legend. Rain is visible while it falls.</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>palette, warm light, diorama orbit 40-62 deg, rain shafts, wet-ground tint, post pass (tilt-shift, grade, vignette). No bloom yet. Screenshots design/look-r12.png, look-r36.png</t>
+        </is>
+      </c>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Readability first, beauty second: a breathing world must show what breathes.</t>
+          <t>Toggle "Diorama" in View compares with/without post. Readability first, beauty second: a breathing world must show what breathes.</t>
         </is>
       </c>
     </row>
@@ -1428,6 +1440,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="6" t="inlineStr">
         <is>
@@ -1449,6 +1462,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="B25" s="6" t="inlineStr">
         <is>
@@ -1511,6 +1525,7 @@
         <v/>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="B32" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Gaia's palette, a diorama orbit, visible rain, and one post pass
One PAL block colours everything: warm limestone rock, cool basalt floor,
ochre rubble, teal water, moss greens, a dusk ground. Warm sun with ACES
tone mapping. Pitch held between 40 and 62 degrees. Rain is a translucent
shaft from ground to cloud; film water darkens and blues the rock it lies
on. A single full-screen shader does tilt-shift, a warm grade and a
vignette, toggled from View as Diorama.

The mechanics sheet records steps 2-4 as done and adds 4b, the player
panel with unlocks, after the first playtest stalled at the first click.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X15nfPExS7vTWJ6rHqpTfb
</commit_message>
<xml_diff>
--- a/design/mechanics.xlsx
+++ b/design/mechanics.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -764,13 +764,13 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>12-hex shore greens over 56 ticks (was 5); alive every 10 ticks 3 5 7 9 11 12</t>
+          <t>12-hex rim full at tick 56 (was 5). LIFE_EVERY=10.</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Commit "Life keeps its own clock". Without this a seed covers the pot in one Season once the world breathes.</t>
+          <t>Without this a seed covers the pot in one Season once the world breathes.</t>
         </is>
       </c>
     </row>
@@ -815,13 +815,13 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>headless: 5 ticks in 2.6 s at 1x, +40 in 2.1 s at 10x, 0 while paused; clock shows Year/Season</t>
+          <t>Runs at 2 ticks/s; 1/3/10/30x; pause; season clock. Headless: 5 ticks in 2.6 s at 1x, 40 in 2.1 s at 10x, 0 paused. Pacing: to be judged in play.</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Mana not yet: actions are free until step 6. Replaces the Moon-per-action idea from design v0.1. Pause is a courtesy, never required.</t>
+          <t>Replaces the Moon-per-action idea from design v0.1. Pause is a courtesy, never required.</t>
         </is>
       </c>
     </row>
@@ -866,33 +866,35 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>palette, warm light, diorama orbit 40-62 deg, rain shafts, wet-ground tint, post pass (tilt-shift, grade, vignette). No bloom yet. Screenshots design/look-r12.png, look-r36.png</t>
+          <t>PAL block, warm sun + ACES, diorama orbit 40-62 deg, rain shafts, wet-ground tint, one post shader (tilt-shift, grade, vignette). No bloom yet. Screenshots in design/.</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Toggle "Diorama" in View compares with/without post. Readability first, beauty second: a breathing world must show what breathes.</t>
+          <t>Readability first, beauty second: a breathing world must show what breathes.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>5</v>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>4b</t>
+        </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Score</t>
+          <t>Onboard</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Harvest: Bloom and Wonders on the bench</t>
+          <t>Player panel and unlocks</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Bloom = living hexes x (1 + sum of Wonder bonuses). A Harvest button shows the arithmetic. No Years yet.</t>
+          <t>The bench panel is hidden behind a "bench" switch. The player sees big buttons only, and earns them: start with DIG alone; RAIN unlocks at the first hollow; SOW unlocks at the first habitable hex; RAISE in Year 2; wider brushes in Year 3. One hint line at a time, triggered by world state, never by a timer.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -900,46 +902,46 @@
           <t>game</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>planned</t>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>next</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Play three boards, try to beat your own Bloom.</t>
+          <t>Hand it to someone who has never seen it. Count seconds to the first click, and to the first seed.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Beating your own number is fun on this sim (go / no-go gate).</t>
+          <t>First click within 10 seconds without asking; a lake and a green shore within 5 minutes; no question "what do I do now".</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>The reversible Step-1 experiment from The Determinism Bet.</t>
+          <t>First playtest (7 Sep): stuck at the first click, "what do we do now?". The panel is a developer bench, not a game.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Score</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Mana</t>
+          <t>Harvest: Bloom and Wonders on the bench</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>10 mana a Year, cost = brush x depth; cloud 3 per rain tile; seed 1; erase cloud/seed 0; rest 0.</t>
+          <t>Bloom = living hexes x (1 + sum of Wonder bonuses). A Harvest button shows the arithmetic. No Years yet.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -954,39 +956,39 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Play a Year with only 10 mana.</t>
+          <t>Play three boards, try to beat your own Bloom.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>A first Year affords: one basin, one cloud, one seed, one hill, a little spare.</t>
+          <t>Beating your own number is fun on this sim (go / no-go gate).</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>See Numbers sheet.</t>
+          <t>The reversible Step-1 experiment from The Determinism Bet.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Loop</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Years, the bar, the pot rests</t>
+          <t>Mana</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>4 Seasons -&gt; Harvest -&gt; Bloom &gt;= target or the run ends on Behold. Targets 8 15 25 40 60 90 130 180.</t>
+          <t>10 mana a Year, cost = brush x depth; cloud 3 per rain tile; seed 1; erase cloud/seed 0; rest 0.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1001,39 +1003,39 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Play three full 8-Year runs.</t>
+          <t>Play a Year with only 10 mana.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Year 5 stalls a count-only build; a shape build clears it.</t>
+          <t>A first Year affords: one basin, one cloud, one seed, one hill, a little spare.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Fail is gentle: no loss, only an ending.</t>
+          <t>See Numbers sheet.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Seed cards: Moss, Grass, Reed</t>
+          <t>Years, the bar, the pot rests</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Deck of 3, hand of 3 per Year, a sown seed spends the card. Each kind is one clause in the habitability rule.</t>
+          <t>4 Seasons -&gt; Harvest -&gt; Bloom &gt;= target or the run ends on Behold. Targets 8 15 25 40 60 90 130 180.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1048,39 +1050,39 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Play with Moss-only, Grass-only, mixed.</t>
+          <t>Play three full 8-Year runs.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>"What to sow" is a real decision; Moss on bare rock reads.</t>
+          <t>Year 5 stalls a count-only build; a shape build clears it.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Willow, Pine, Lotus later (step 12).</t>
+          <t>Fail is gentle: no loss, only an ending.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Shop</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Spring shop, Dew, six Boons</t>
+          <t>Seed cards: Moss, Grass, Reed</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Dew = 2 + surplus/5 (cap 10) + interest. 3 Boons + 2 seeds offered, reroll 2. First six: Monsoon, Wellspring, Long Summer, Deep Roots, Basalt Heart, Lake Heart.</t>
+          <t>Deck of 3, hand of 3 per Year, a sown seed spends the card. Each kind is one clause in the habitability rule.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1095,39 +1097,39 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Play three runs aiming at Lake / River / Highland.</t>
+          <t>Play with Moss-only, Grass-only, mixed.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Two runs feel different because of the shop, not the dice.</t>
+          <t>"What to sow" is a real decision; Moss on bare rock reads.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Offers come from the run seed.</t>
+          <t>Willow, Pine, Lotus later (step 12).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Variety</t>
+          <t>Shop</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Seeded starting pots</t>
+          <t>Spring shop, Dew, six Boons</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>A seed number makes the starting shape (hills, a hollow, rubble) and every shop. No randomness after the run begins.</t>
+          <t>Dew = 2 + surplus/5 (cap 10) + interest. 3 Boons + 2 seeds offered, reroll 2. First six: Monsoon, Wellspring, Long Summer, Deep Roots, Basalt Heart, Lake Heart.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1142,39 +1144,39 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Same seed twice; different seeds five times.</t>
+          <t>Play three runs aiming at Lake / River / Highland.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Identical runs from one seed; distinct openings from five.</t>
+          <t>Two runs feel different because of the shop, not the dice.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr"/>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Daily seed for free.</t>
+          <t>Offers come from the run seed.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Wheel</t>
+          <t>Variety</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Gaia's Whim (the wheel)</t>
+          <t>Seeded starting pots</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Earned, never scheduled: fires on a milestone (e.g. 30% of the pot under water, a peak at height 8, first Ring of Life). The wheel picks a FORCE from the run seed; the player AIMS it. Forces never score; they only change the world.</t>
+          <t>A seed number makes the starting shape (hills, a hollow, rubble) and every shop. No randomness after the run begins.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1184,44 +1186,44 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>idea</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Prototype with three forces: Meteor (crater + slag ring), Megatime (100 ticks in 5 s), Monsoon (clouds x2 for a Season).</t>
+          <t>Same seed twice; different seeds five times.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>It feels like a reward, not a tax; the best play is still shaping, never fishing for spins.</t>
+          <t>Identical runs from one seed; distinct openings from five.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>See Wheel sheet. Kept OUT of the core loop and OUT of scoring. Frequency target: 2-3 a run.</t>
+          <t>Daily seed for free.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Wheel</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Willow, Pine, Lotus</t>
+          <t>Gaia's Whim (the wheel)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Bank-only fast spreader; highland slow tree worth 2; still-water plant.</t>
+          <t>Earned, never scheduled: fires on a milestone (e.g. 30% of the pot under water, a peak at height 8, first Ring of Life). The wheel picks a FORCE from the run seed; the player AIMS it. Forces never score; they only change the world.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1231,44 +1233,44 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>idea</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>One run built around each.</t>
+          <t>Prototype with three forces: Meteor (crater + slag ring), Megatime (100 ticks in 5 s), Monsoon (clouds x2 for a Season).</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Each opens a build the others do not.</t>
+          <t>It feels like a reward, not a tax; the best play is still shaping, never fishing for spins.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Lotus needs "alive on water" which is one clause, not a system.</t>
+          <t>See Wheel sheet. Kept OUT of the core loop and OUT of scoring. Frequency target: 2-3 a run.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Shop</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Remaining Boons</t>
+          <t>Willow, Pine, Lotus</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Beaver, Silt, Terraces, Migrating Birds, Gaia's Patience; Old Growth last (needs age state).</t>
+          <t>Bank-only fast spreader; highland slow tree worth 2; still-water plant.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1283,39 +1285,39 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Add two at a time; play.</t>
+          <t>One run built around each.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>No Boon is a must-buy; no Boon is dead.</t>
+          <t>Each opens a build the others do not.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Old Growth is the only one adding stored state.</t>
+          <t>Lotus needs "alive on water" which is one clause, not a system.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Cozy</t>
+          <t>Shop</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Cozy mode, Codex, Requests</t>
+          <t>Remaining Boons</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>No bar, no clock pressure, 20 mana carried, shop as a menu, Wonders as a notebook, optional Requests.</t>
+          <t>Beaver, Silt, Terraces, Migrating Birds, Gaia's Patience; Old Growth last (needs age state).</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1330,44 +1332,44 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Hand it to someone who does not play roguelikes.</t>
+          <t>Add two at a time; play.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>They stay 20 minutes and take a screenshot.</t>
+          <t>No Boon is a must-buy; no Boon is dead.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>A mode, not the spine.</t>
+          <t>Old Growth is the only one adding stored state.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Payoff</t>
+          <t>Cozy</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Behold</t>
+          <t>Cozy mode, Codex, Requests</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>End of run: the diorama, photo mode, the run's story (Wonders found, Bloom per Year).</t>
+          <t>No bar, no clock pressure, 20 mana carried, shop as a menu, Wonders as a notebook, optional Requests.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>presentation</t>
+          <t>game</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1377,44 +1379,44 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Show a stranger the screen.</t>
+          <t>Hand it to someone who does not play roguelikes.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>"I want to try".</t>
+          <t>They stay 20 minutes and take a screenshot.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>The trailer's last shot.</t>
+          <t>A mode, not the spine.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Ship</t>
+          <t>Payoff</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Vertical slice -&gt; demo</t>
+          <t>Behold</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Fixed teaching pot for Year 1, capsule, GIF, Steam page, Next Fest.</t>
+          <t>End of run: the diorama, photo mode, the run's story (Wonders found, Bloom per Year).</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>ship</t>
+          <t>presentation</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1424,136 +1426,180 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Next Fest wishlists.</t>
+          <t>Show a stranger the screen.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>7k+ wishlists (Popular Upcoming threshold).</t>
+          <t>"I want to try".</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr"/>
       <c r="J19" s="4" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr">
         <is>
+          <t>The trailer's last shot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Ship</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Vertical slice -&gt; demo</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Fixed teaching pot for Year 1, capsule, GIF, Steam page, Next Fest.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>ship</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Next Fest wishlists.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>7k+ wishlists (Popular Upcoming threshold).</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
           <t>Steam-first, ~$13.</t>
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="B21" s="6" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Legend</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Yellow cells are for you to fill in after a playtest: Result, and Decision (keep / tune / cut).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="7" t="inlineStr">
         <is>
+          <t>Yellow cells are for you to fill in after a playtest: Result, and Decision (keep / tune / cut).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
           <t>One step at a time: nothing in a later row starts until the row above has a Result and a Decision.</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="B25" s="6" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="C26" s="7">
-        <f>COUNTIF($F$2:$F$19,B26)</f>
-        <v/>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>next</t>
+          <t>done</t>
         </is>
       </c>
       <c r="C27" s="7">
-        <f>COUNTIF($F$2:$F$19,B27)</f>
+        <f>COUNTIF($F$2:$F$20,B27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>next</t>
         </is>
       </c>
       <c r="C28" s="7">
-        <f>COUNTIF($F$2:$F$19,B28)</f>
+        <f>COUNTIF($F$2:$F$20,B28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>idea</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="C29" s="7">
-        <f>COUNTIF($F$2:$F$19,B29)</f>
+        <f>COUNTIF($F$2:$F$20,B29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="7" t="inlineStr">
         <is>
+          <t>idea</t>
+        </is>
+      </c>
+      <c r="C30" s="7">
+        <f>COUNTIF($F$2:$F$20,B30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
           <t>cut</t>
         </is>
       </c>
-      <c r="C30" s="7">
-        <f>COUNTIF($F$2:$F$19,B30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>decided</t>
-        </is>
-      </c>
-      <c r="C32" s="7">
-        <f>COUNTA($J$2:$J$19)</f>
+      <c r="C31" s="7">
+        <f>COUNTIF($F$2:$F$20,B31)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="7" t="inlineStr">
         <is>
+          <t>decided</t>
+        </is>
+      </c>
+      <c r="C33" s="7">
+        <f>COUNTA($J$2:$J$20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="7" t="inlineStr">
+        <is>
           <t>kept</t>
         </is>
       </c>
-      <c r="C33" s="7">
-        <f>COUNTIF($J$2:$J$19,"keep")</f>
+      <c r="C34" s="7">
+        <f>COUNTIF($J$2:$J$20,"keep")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="F2:F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"done,next,planned,idea,cut"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"keep,tune,cut"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3572,7 +3618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3678,6 +3724,51 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>steps (2-3)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>2 - Life clock, 3 - Breathing world</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>partner + founder</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Opened the page: "what do we do now?". Stuck at the first click. Panel felt like it needs a PC-game expert.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Confusing. The world is fine; the panel is not a game.</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>tune</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>4b: player panel + unlocks, one hint at a time</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Player mode: powers are earned, and one file to send
The page opens as a game: a pot of rock, a dock of big buttons, one hint.
Tools unlock from the world's own state -- rain at the first hollow, speed
at the first water tile, sow at the first habitable hex, raise at the first
living hex -- never on a timer. A one-word tip by the pointer says why a
seed would not take. TR and EN. The bench is behind the corner button and
?bench=1.

build.js folds three.js into pot.html so it opens from a double click.
Verified headless from file://: the whole chain, no errors.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X15nfPExS7vTWJ6rHqpTfb
</commit_message>
<xml_diff>
--- a/design/mechanics.xlsx
+++ b/design/mechanics.xlsx
@@ -47,7 +47,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,11 +67,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEFD6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4E6CF"/>
       </patternFill>
     </fill>
   </fills>
@@ -101,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -113,9 +108,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -485,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -902,9 +894,9 @@
           <t>game</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>next</t>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -917,7 +909,11 @@
           <t>First click within 10 seconds without asking; a lake and a green shore within 5 minutes; no question "what do I do now".</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Built: dock of big buttons, one hint line, one-word tip by the pointer, TR/EN, bench behind a corner button. Chain checked headless: dig -&gt; rain -&gt; wait -&gt; sow -&gt; raise, shore habitable at tick ~100 (0.7 u/tick). pot.html is a single file that opens by double click. Seconds-to-first-click: YOUR test.</t>
+        </is>
+      </c>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -926,69 +922,75 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>5</v>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>4c</t>
+        </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Score</t>
+          <t>Ship</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Harvest: Bloom and Wonders on the bench</t>
+          <t>One file to send</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Bloom = living hexes x (1 + sum of Wonder bonuses). A Harvest button shows the arithmetic. No Years yet.</t>
+          <t>node build.js folds three.js into the page: pot.html opens from a double click, no server, and can be sent over a chat.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>game</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>planned</t>
+          <t>ship</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Play three boards, try to beat your own Bloom.</t>
+          <t>Open pot.html from a chat download on a machine with no repo.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Beating your own number is fun on this sim (go / no-go gate).</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr"/>
+          <t>It opens and plays.</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Verified headless from file://. Rebuild after every change to index.html.</t>
+        </is>
+      </c>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>The reversible Step-1 experiment from The Determinism Bet.</t>
+          <t>Bench stays index.html + run.bat.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Score</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Mana</t>
+          <t>Harvest: Bloom and Wonders on the bench</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>10 mana a Year, cost = brush x depth; cloud 3 per rain tile; seed 1; erase cloud/seed 0; rest 0.</t>
+          <t>Bloom = living hexes x (1 + sum of Wonder bonuses). A Harvest button shows the arithmetic. No Years yet.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1003,39 +1005,39 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Play a Year with only 10 mana.</t>
+          <t>Play three boards, try to beat your own Bloom.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>A first Year affords: one basin, one cloud, one seed, one hill, a little spare.</t>
+          <t>Beating your own number is fun on this sim (go / no-go gate).</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>See Numbers sheet.</t>
+          <t>The reversible Step-1 experiment from The Determinism Bet.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Loop</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Years, the bar, the pot rests</t>
+          <t>Mana</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>4 Seasons -&gt; Harvest -&gt; Bloom &gt;= target or the run ends on Behold. Targets 8 15 25 40 60 90 130 180.</t>
+          <t>10 mana a Year, cost = brush x depth; cloud 3 per rain tile; seed 1; erase cloud/seed 0; rest 0.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1050,39 +1052,39 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Play three full 8-Year runs.</t>
+          <t>Play a Year with only 10 mana.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Year 5 stalls a count-only build; a shape build clears it.</t>
+          <t>A first Year affords: one basin, one cloud, one seed, one hill, a little spare.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Fail is gentle: no loss, only an ending.</t>
+          <t>See Numbers sheet.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Seed cards: Moss, Grass, Reed</t>
+          <t>Years, the bar, the pot rests</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Deck of 3, hand of 3 per Year, a sown seed spends the card. Each kind is one clause in the habitability rule.</t>
+          <t>4 Seasons -&gt; Harvest -&gt; Bloom &gt;= target or the run ends on Behold. Targets 8 15 25 40 60 90 130 180.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1097,39 +1099,39 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Play with Moss-only, Grass-only, mixed.</t>
+          <t>Play three full 8-Year runs.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>"What to sow" is a real decision; Moss on bare rock reads.</t>
+          <t>Year 5 stalls a count-only build; a shape build clears it.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Willow, Pine, Lotus later (step 12).</t>
+          <t>Fail is gentle: no loss, only an ending.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Shop</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Spring shop, Dew, six Boons</t>
+          <t>Seed cards: Moss, Grass, Reed</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Dew = 2 + surplus/5 (cap 10) + interest. 3 Boons + 2 seeds offered, reroll 2. First six: Monsoon, Wellspring, Long Summer, Deep Roots, Basalt Heart, Lake Heart.</t>
+          <t>Deck of 3, hand of 3 per Year, a sown seed spends the card. Each kind is one clause in the habitability rule.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1144,39 +1146,39 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Play three runs aiming at Lake / River / Highland.</t>
+          <t>Play with Moss-only, Grass-only, mixed.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Two runs feel different because of the shop, not the dice.</t>
+          <t>"What to sow" is a real decision; Moss on bare rock reads.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr"/>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Offers come from the run seed.</t>
+          <t>Willow, Pine, Lotus later (step 12).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Variety</t>
+          <t>Shop</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Seeded starting pots</t>
+          <t>Spring shop, Dew, six Boons</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>A seed number makes the starting shape (hills, a hollow, rubble) and every shop. No randomness after the run begins.</t>
+          <t>Dew = 2 + surplus/5 (cap 10) + interest. 3 Boons + 2 seeds offered, reroll 2. First six: Monsoon, Wellspring, Long Summer, Deep Roots, Basalt Heart, Lake Heart.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1191,39 +1193,39 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Same seed twice; different seeds five times.</t>
+          <t>Play three runs aiming at Lake / River / Highland.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Identical runs from one seed; distinct openings from five.</t>
+          <t>Two runs feel different because of the shop, not the dice.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Daily seed for free.</t>
+          <t>Offers come from the run seed.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Wheel</t>
+          <t>Variety</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Gaia's Whim (the wheel)</t>
+          <t>Seeded starting pots</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Earned, never scheduled: fires on a milestone (e.g. 30% of the pot under water, a peak at height 8, first Ring of Life). The wheel picks a FORCE from the run seed; the player AIMS it. Forces never score; they only change the world.</t>
+          <t>A seed number makes the starting shape (hills, a hollow, rubble) and every shop. No randomness after the run begins.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1233,44 +1235,44 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>idea</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Prototype with three forces: Meteor (crater + slag ring), Megatime (100 ticks in 5 s), Monsoon (clouds x2 for a Season).</t>
+          <t>Same seed twice; different seeds five times.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>It feels like a reward, not a tax; the best play is still shaping, never fishing for spins.</t>
+          <t>Identical runs from one seed; distinct openings from five.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>See Wheel sheet. Kept OUT of the core loop and OUT of scoring. Frequency target: 2-3 a run.</t>
+          <t>Daily seed for free.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Wheel</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Willow, Pine, Lotus</t>
+          <t>Gaia's Whim (the wheel)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Bank-only fast spreader; highland slow tree worth 2; still-water plant.</t>
+          <t>Earned, never scheduled: fires on a milestone (e.g. 30% of the pot under water, a peak at height 8, first Ring of Life). The wheel picks a FORCE from the run seed; the player AIMS it. Forces never score; they only change the world.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1280,44 +1282,44 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>idea</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>One run built around each.</t>
+          <t>Prototype with three forces: Meteor (crater + slag ring), Megatime (100 ticks in 5 s), Monsoon (clouds x2 for a Season).</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Each opens a build the others do not.</t>
+          <t>It feels like a reward, not a tax; the best play is still shaping, never fishing for spins.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Lotus needs "alive on water" which is one clause, not a system.</t>
+          <t>See Wheel sheet. Kept OUT of the core loop and OUT of scoring. Frequency target: 2-3 a run.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Shop</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Remaining Boons</t>
+          <t>Willow, Pine, Lotus</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Beaver, Silt, Terraces, Migrating Birds, Gaia's Patience; Old Growth last (needs age state).</t>
+          <t>Bank-only fast spreader; highland slow tree worth 2; still-water plant.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1332,39 +1334,39 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Add two at a time; play.</t>
+          <t>One run built around each.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>No Boon is a must-buy; no Boon is dead.</t>
+          <t>Each opens a build the others do not.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Old Growth is the only one adding stored state.</t>
+          <t>Lotus needs "alive on water" which is one clause, not a system.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Cozy</t>
+          <t>Shop</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Cozy mode, Codex, Requests</t>
+          <t>Remaining Boons</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>No bar, no clock pressure, 20 mana carried, shop as a menu, Wonders as a notebook, optional Requests.</t>
+          <t>Beaver, Silt, Terraces, Migrating Birds, Gaia's Patience; Old Growth last (needs age state).</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1379,44 +1381,44 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Hand it to someone who does not play roguelikes.</t>
+          <t>Add two at a time; play.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>They stay 20 minutes and take a screenshot.</t>
+          <t>No Boon is a must-buy; no Boon is dead.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>A mode, not the spine.</t>
+          <t>Old Growth is the only one adding stored state.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Payoff</t>
+          <t>Cozy</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Behold</t>
+          <t>Cozy mode, Codex, Requests</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>End of run: the diorama, photo mode, the run's story (Wonders found, Bloom per Year).</t>
+          <t>No bar, no clock pressure, 20 mana carried, shop as a menu, Wonders as a notebook, optional Requests.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>presentation</t>
+          <t>game</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1426,44 +1428,44 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Show a stranger the screen.</t>
+          <t>Hand it to someone who does not play roguelikes.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>"I want to try".</t>
+          <t>They stay 20 minutes and take a screenshot.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr"/>
       <c r="J19" s="4" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>The trailer's last shot.</t>
+          <t>A mode, not the spine.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Ship</t>
+          <t>Payoff</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Vertical slice -&gt; demo</t>
+          <t>Behold</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Fixed teaching pot for Year 1, capsule, GIF, Steam page, Next Fest.</t>
+          <t>End of run: the diorama, photo mode, the run's story (Wonders found, Bloom per Year).</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>ship</t>
+          <t>presentation</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1473,133 +1475,180 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Next Fest wishlists.</t>
+          <t>Show a stranger the screen.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>7k+ wishlists (Popular Upcoming threshold).</t>
+          <t>"I want to try".</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
+          <t>The trailer's last shot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Ship</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Vertical slice -&gt; demo</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Fixed teaching pot for Year 1, capsule, GIF, Steam page, Next Fest.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>ship</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Next Fest wishlists.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>7k+ wishlists (Popular Upcoming threshold).</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
           <t>Steam-first, ~$13.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="6" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="7" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Yellow cells are for you to fill in after a playtest: Result, and Decision (keep / tune / cut).</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="7" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>One step at a time: nothing in a later row starts until the row above has a Result and a Decision.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="6" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="7" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="C27" s="7">
-        <f>COUNTIF($F$2:$F$20,B27)</f>
+      <c r="C28" s="6">
+        <f>COUNTIF($F$2:$F$21,B28)</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="7" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>next</t>
         </is>
       </c>
-      <c r="C28" s="7">
-        <f>COUNTIF($F$2:$F$20,B28)</f>
+      <c r="C29" s="6">
+        <f>COUNTIF($F$2:$F$21,B29)</f>
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="7" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="C29" s="7">
-        <f>COUNTIF($F$2:$F$20,B29)</f>
+      <c r="C30" s="6">
+        <f>COUNTIF($F$2:$F$21,B30)</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="7" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>idea</t>
         </is>
       </c>
-      <c r="C30" s="7">
-        <f>COUNTIF($F$2:$F$20,B30)</f>
+      <c r="C31" s="6">
+        <f>COUNTIF($F$2:$F$21,B31)</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="7" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>cut</t>
         </is>
       </c>
-      <c r="C31" s="7">
-        <f>COUNTIF($F$2:$F$20,B31)</f>
+      <c r="C32" s="6">
+        <f>COUNTIF($F$2:$F$21,B32)</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="7" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>decided</t>
         </is>
       </c>
-      <c r="C33" s="7">
-        <f>COUNTA($J$2:$J$20)</f>
+      <c r="C34" s="6">
+        <f>COUNTA($J$2:$J$21)</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="7" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>kept</t>
         </is>
       </c>
-      <c r="C34" s="7">
-        <f>COUNTIF($J$2:$J$20,"keep")</f>
+      <c r="C35" s="6">
+        <f>COUNTIF($J$2:$J$21,"keep")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="F2:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"done,next,planned,idea,cut"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"keep,tune,cut"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2607,27 +2656,27 @@
       <c r="F13" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Sum of all bonuses</t>
         </is>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="6">
         <f>SUM(D2:D13)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Example: 22 living hexes with Lake + River + Ring</t>
         </is>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="6">
         <f>22*(1+D2+D4+D9)</f>
         <v/>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Bloom</t>
         </is>

</xml_diff>

<commit_message>
The sheet: step 5 done, Wonder results, English only
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X15nfPExS7vTWJ6rHqpTfb
</commit_message>
<xml_diff>
--- a/design/mechanics.xlsx
+++ b/design/mechanics.xlsx
@@ -911,7 +911,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Built: dock of big buttons, one hint line, one-word tip by the pointer, TR/EN, bench behind a corner button. Chain checked headless: dig -&gt; rain -&gt; wait -&gt; sow -&gt; raise, shore habitable at tick ~100 (0.7 u/tick). pot.html is a single file that opens by double click. Seconds-to-first-click: YOUR test.</t>
+          <t>Built: dock of big buttons, one hint line, one-word tip by the pointer, English only, bench behind a corner button. Chain checked headless: dig -&gt; rain -&gt; wait -&gt; sow -&gt; raise, shore habitable at tick ~100 (0.7 u/tick). pot.html is a single file that opens by double click. Seconds-to-first-click: YOUR test.</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr"/>
@@ -998,9 +998,9 @@
           <t>game</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>planned</t>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1013,7 +1013,11 @@
           <t>Beating your own number is fun on this sim (go / no-go gate).</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>12 detectors in the core, pure reads; Harvest screen at every Year turn with the arithmetic and the Codex; harvest button on the bench. Seeded bowl: Lake+Ring+Grove = 12 x 2.75 = 33. wonders() at radius 64: 14 ms. Fun: YOUR test.</t>
+        </is>
+      </c>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -2389,7 +2393,11 @@
       <c r="E2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>detects on the seeded bowl</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2413,7 +2421,11 @@
       <c r="E3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>detects on a moat</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2437,7 +2449,11 @@
       <c r="E4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>detects on a trench; the flow pulses 65/13 tile by tile, the walk allows one quiet tile</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2461,7 +2477,11 @@
       <c r="E5" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>detects on a stepped trench</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2485,7 +2505,11 @@
       <c r="E6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>needs more than one cloud to clear the bar both ways: tune</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2509,7 +2533,11 @@
       <c r="E7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>not yet seen on a test board</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2533,7 +2561,11 @@
       <c r="E8" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>detects on a moat</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2557,7 +2589,11 @@
       <c r="E9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>detects on the seeded bowl</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2581,7 +2617,11 @@
       <c r="E10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>detects</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2605,7 +2645,11 @@
       <c r="E11" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>detects on a cone</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2629,7 +2673,11 @@
       <c r="E12" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>detects on a cone</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2653,7 +2701,11 @@
       <c r="E13" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>detects on a split channel</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">

</xml_diff>

<commit_message>
The sheet records the first playable block
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X15nfPExS7vTWJ6rHqpTfb
</commit_message>
<xml_diff>
--- a/design/mechanics.xlsx
+++ b/design/mechanics.xlsx
@@ -1049,9 +1049,9 @@
           <t>game</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>planned</t>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1064,7 +1064,11 @@
           <t>A first Year affords: one basin, one cloud, one seed, one hill, a little spare.</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>10 mana a Year; Dig 2, Raise 2, Rain 3, Sow 1; a cloud clicked again is taken away for nothing. Tools grey out when unaffordable. Checked in the browser: dig+rain 10-&gt;5, sow -&gt;4, a fifth click refused.</t>
+        </is>
+      </c>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1096,9 +1100,9 @@
           <t>game</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>planned</t>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1111,7 +1115,11 @@
           <t>Year 5 stalls a count-only build; a shape build clears it.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Targets 8 15 25 40 60 90 130 180. Harvest against the target at the turn of the Year; miss -&gt; The pot rests (Behold); Year 8 cleared -&gt; A world. Idle pot rests at Year 1 with Bloom 0. Dew = 2 + surplus/5 (cap 10) + interest.</t>
+        </is>
+      </c>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1143,9 +1151,9 @@
           <t>game</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>planned</t>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1158,7 +1166,11 @@
           <t>"What to sow" is a real decision; Moss on bare rock reads.</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Grass, Moss (bare rock, worth half), Reed (one tile deep). Deck starts Grass Grass Moss; hand = deck each Year; a sown seed spends a card. Kinds spread as what they are: GGGGmGmmmmmm on a half-soiled rim.</t>
+        </is>
+      </c>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -1190,9 +1202,9 @@
           <t>game</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>planned</t>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1205,7 +1217,11 @@
           <t>Two runs feel different because of the shop, not the dice.</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Spring after every cleared Year: 3 Boons + 2 seed cards from the run seed, reroll 2 dew, max 5 Boons. Six Boons: Monsoon, Wellspring, Long Summer, Deep Roots, Basalt Heart, Lake Heart. Bought Monsoon in the browser run; rain x1.5 verified headless.</t>
+        </is>
+      </c>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1284,9 +1300,9 @@
           <t>game</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>idea</t>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1299,7 +1315,11 @@
           <t>It feels like a reward, not a tax; the best play is still shaping, never fishing for spins.</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Gaia's Whim fires on the first Lake, first River, first Ring of Life; the wheel runs round and slows onto a force from the run seed: Meteor (aimed: crater r2, two steps, slag ring), Megatime (100 ticks in ~2.5 s), Monsoon (rain x2 for a Season). Never scores. Fired on the first Lake in the browser run and gave Monsoon.</t>
+        </is>
+      </c>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
The sheet and the handoff record steps 12 to 19
Steps rows 22-29 for the meteor VFX, the wheel opening up, the eight forces,
the sow-unlock bug, the readout and panel, the Codex recipes, tilt-shift and
Omens -- each with what was measured. The summary COUNTIFs were reading
$F$2:$F$21 and the data block was already full to 21, so the ranges are
widened to $F$2:$F$29 rather than the rows being dropped past them.

A new Omens sheet: the four shapes, what each reads from harvest(), how the
dew scales, and how the pool grows with the Year. The Wheel sheet gains a
BUILT block saying which proposals were taken (Quake became Upheaval, Seed
Rain was not built) and answers the risk noted in its own row 14 -- the
meteor crater is bare bedrock, so it makes a basin faster than digging but
gives no soil in the middle, and digging is still wanted.

Playtest log: the first full run, the Moss report and its cause, and the
pending fourth test.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design/mechanics.xlsx
+++ b/design/mechanics.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Steps" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Numbers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Wonders" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Seeds" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Boons" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Wheel" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Playtest log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numbers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wonders" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seeds" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boons" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wheel" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Omens" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Playtest log" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -96,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -112,6 +113,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -477,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1562,108 +1566,535 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Meteor VFX</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>A meteor you can watch land</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>The crater rule is unchanged; a bolide falls for 0.9 s, then flash, camera shake and an expanding ring.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Step fx() against a fake clock at 60 fps and read the whole timeline.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>The crater applies exactly at impact, everything resets, and a hidden tab returns to a finished crater.</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>bolide y 18.83-&gt;0.34 over 0.90 s; h 1-&gt;-1; flash peak 0.95 gone by 1.27; shake 0.94; ring 0.71-&gt;8.1; all reset by 3.10</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Timed off the wall clock, not accumulated frame deltas: clamped deltas made the fall take 6 s at 10 fps.</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="B23" s="5" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Whim</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Every Wonder turns the wheel</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Each of the twelve Wonders turns the wheel the first time it stands in this run.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Count how many wheels a run can give, and when they land.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Wheels spread over the run instead of all landing by Year 3.</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>was 3 milestones, all firsts, all before Year 3; now up to 12, with the hard Wonders arriving late</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>No new state: RUN.whims was already keyed by name. Still earned, still never scheduled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Whim</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Eight forces, in three shapes</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Spells (a Season, reversible), Aimed (one tick, one hex), Instant. Only levers the sim already has.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Land each aimed force on a flat pot; turn all three spells on and off.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Each force does exactly what its line says; the spells restore their levers exactly.</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Upheaval h 3/3/2/1 by distance; Landslide 6/4/2/0 courses; Cloudburst 10.29/6.29/2.00/4.00 after a tick; spells on 2 / 2.8 / 1, off 1 / 0.7 / 10 exact</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Refiring a running spell extends it rather than stacking it, which is what keeps the multiplicative off() exact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Sow unlocks for any seed in the hand</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>The unlock ladder asks about every seed held, not only Grass.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Hand-dug hollow with water in it, weathering 0.7 a tick: when does sow appear?</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>The tool appears while a seed in the deck would take.</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Grass only: tick 100. Any seed held: tick 1. This was the "I can never sow Moss" report.</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>A real bug, not a presentation gap. A hand-dug pot has bare rock walls and no slag at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>The screen says what is going on</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>The tip names the ground and the seed that would take; the panel carries mana, Boons, running forces and the deck.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Hover a bare rock shore while holding Grass; fill a run with Boons and a spell.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>It names the alternative rather than only refusing, and nothing held is invisible.</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>"rock / bare - Moss takes here"; panel reads 4/10 mana with Monsoon, Basalt Heart, Ages of Frost 120 ticks, Grass x2, Moss x1</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Answers four separate playtest complaints at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>The Codex says how a Wonder is made</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Each of the twelve carries a one-line recipe restated from its detector; a button opens it during play.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Read every recipe against the detector it describes.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Every line is true to the code.</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>12 of 12 match; the grid shows recipes whether or not the Wonder was found; opens from the play HUD</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>From the playtest: "how is a Wonder made? I do not know how we would get one."</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Look</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Tilt-shift you can actually see</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Two-pass separable blur, nine taps each way, masked by a band in screen space.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Mean absolute horizontal gradient of the final framebuffer, by screen band.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>The near skirt softens and the focus band does not.</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>detail lost at the bottom of the frame: 16.0% as it was, 29.8% at the new default, 41.4% at 12 px; inside the focus band 0.0 / 1.0 / 1.6%</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>On a slider, the same reasoning as WEATHER: no calibration for it exists yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Omens</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>The Year asks for one thing</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Three Omens offered at the turn of the Year and one chosen; read from the same Harvest; pays dew.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Generate the pool for all eight Years; harvest with the Omen met and with it missed.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>The pool grows with the Year and both branches pay correctly.</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>pool 8 / 14 / 18 across the run; Year 1 "The Lake stands +4", Year 8 "3 Deltas at once +12"; met pays +3 dew (0-&gt;3), missed pays nothing</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>No new state, no new detector, nothing random after the run seed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Yellow cells are for you to fill in after a playtest: Result, and Decision (keep / tune / cut).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>One step at a time: nothing in a later row starts until the row above has a Result and a Decision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="C28" s="6">
-        <f>COUNTIF($F$2:$F$21,B28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>next</t>
-        </is>
-      </c>
-      <c r="C29" s="6">
-        <f>COUNTIF($F$2:$F$21,B29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="C30" s="6">
-        <f>COUNTIF($F$2:$F$21,B30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>idea</t>
-        </is>
-      </c>
-      <c r="C31" s="6">
-        <f>COUNTIF($F$2:$F$21,B31)</f>
-        <v/>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="6" t="inlineStr">
         <is>
+          <t>Yellow cells are for you to fill in after a playtest: Result, and Decision (keep / tune / cut).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>One step at a time: nothing in a later row starts until the row above has a Result and a Decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="C36" s="6">
+        <f>COUNTIF($F$2:$F$29,B28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>next</t>
+        </is>
+      </c>
+      <c r="C37" s="6">
+        <f>COUNTIF($F$2:$F$29,B29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="C38" s="6">
+        <f>COUNTIF($F$2:$F$29,B30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>idea</t>
+        </is>
+      </c>
+      <c r="C39" s="6">
+        <f>COUNTIF($F$2:$F$29,B31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="6" t="inlineStr">
+        <is>
           <t>cut</t>
         </is>
       </c>
-      <c r="C32" s="6">
-        <f>COUNTIF($F$2:$F$21,B32)</f>
+      <c r="C40" s="6">
+        <f>COUNTIF($F$2:$F$29,B32)</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="6" t="inlineStr">
+    <row r="41"/>
+    <row r="42">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>decided</t>
         </is>
       </c>
-      <c r="C34" s="6">
-        <f>COUNTA($J$2:$J$21)</f>
+      <c r="C42" s="6">
+        <f>COUNTA($J$2:$J$29)</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="6" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>kept</t>
         </is>
       </c>
-      <c r="C35" s="6">
-        <f>COUNTIF($J$2:$J$21,"keep")</f>
+      <c r="C43" s="6">
+        <f>COUNTIF($J$2:$J$29,"keep")</f>
         <v/>
       </c>
     </row>
@@ -3435,7 +3866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3725,6 +4156,226 @@
       <c r="D14" s="2" t="inlineStr">
         <is>
           <t>measure in step 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: when it appears</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>every Wonder, the first time it stands this run (12 of them)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>the three firsts all landed in Year 1-2; every Wonder spreads the wheel over the whole run</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>replaces the 3-milestone proposal in row 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: the shortlist</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>three of the eight, drawn from the run seed</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>all eight was a wall of text and made every wheel look the same</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: Force Meteor</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>crater 2 steps deep over r2, slag ring at r3, with a falling bolide</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>the rule is unchanged; it is now visible</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: Force Upheaval</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>the ground swells 2 steps at r0-1 and 1 step at r2</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>the mirror of Meteor; replaces the "Quake" proposal</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: Force Landslide</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>6, 4, 2 courses of slag at r0, r1, r2</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>loose material the water then sorts</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: Force Cloudburst</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>12 courses of water over r2, all at once</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>a lake handed to you, which then has to drain</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: Force Monsoon</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>twice the rain for one Season</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>RAIN_MULT, exactly reversible</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: Force Ages of Frost</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>rock breaks down four times as fast, one Season</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>WEATHER, exactly reversible</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: Force Quickening</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>life steps every tick instead of every tenth, one Season</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>LIFE_EVERY, exactly reversible</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>BUILT: Force Megatime</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>a hundred ticks in a breath</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>unchanged from the proposal</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>NOT built: Seed Rain</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>still on the table</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Risk from row 14, looked at</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>the meteor crater is bare bedrock ringed by slag</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>it makes a basin faster than digging, but the middle has no soil, so digging is still wanted</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>watch it in the next playtest</t>
         </is>
       </c>
     </row>
@@ -3739,7 +4390,313 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Shape</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Read from harvest()</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Dew</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Years offered</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Result (fill in)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Decision (keep / tune / cut)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>stands</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>"The Lake stands."</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>h.wonders[k]</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>2 + 4 x BONUS[k]</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr"/>
+      <c r="G2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>many</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>"3 Deltas at once."</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>h.wonders[k] &gt;= n</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>3 + 4 x BONUS[k] x n</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>all; n is 2 early, 3 late</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>living</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>"40 living hexes."</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>h.alive &gt;= n</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>2 + n/8</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>all; n is 8 / 20 / 40 by Year</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>variety</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>"3 different Wonders at once."</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>keys(h.wonders).length &gt;= n</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>3 + 2n</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>all; n is 2 / 3 / 4 by Year</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>pool, Years 1-2</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>the easy Wonders only</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Lake, River, Waterfall, Grove</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>8 entries</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>pool, Years 3-5</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>and the middling ones</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>+ Great Lake, Fork, Island, Terrace, Highland Meadow</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>14 entries</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>pool, Years 6-8</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>and the hard ones</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>+ Delta, Ring of Life, Watershed</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>18 entries</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr"/>
+      <c r="G8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>the choice</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>three offered, one taken, or None this Year</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>a goal you picked is a plan; a goal handed to you is a chore</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>when it pays</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>at the Harvest, whether or not the target was cleared</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>open question</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>is dew the right reward, or should a met Omen turn the wheel instead?</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3890,6 +4847,131 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>8a9f776</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>First full run, steps 1-11</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>founder</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>one run</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Played the first playable end to end. The core mechanic is liked. The wheel came too seldom; no quest ever arrives; nothing new turns up in the later Years; the meteor landed invisibly.</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>The loop is right and the run is front-loaded: everything the game has arrives in Year 1-2.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>tune</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Measured it: 3 wheels, all before Year 3; Boon offers 3/3/3/3/2/1/1; 4 verbs all unlocked in Year 1. Built steps 12-19 in answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>d6a1e2f</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>founder</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Reported: "I can never sow Moss anywhere."</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Read as a design problem. It was a bug.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Sow unlocked only when a hex was habitable for GRASS, which needs a course of soil. A hand-dug pot is bare rock, so on those boards the tool appeared at tick 100 instead of tick 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>95707d8</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Steps 12-19</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Next: the founder plays a run on the new build and says whether the later Years now have something in them.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>